<commit_message>
Conexão com banco de dados e arquivos do projeto
</commit_message>
<xml_diff>
--- a/Planilha de requisitos.xlsx
+++ b/Planilha de requisitos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Projetos de sistemas microprocessados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B467B01-5BB3-4D49-BBF0-3D2A16F78076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CD27D0-5427-4F56-B729-7E4DF9E6BCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,12 +401,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -417,7 +411,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,145 +709,145 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="7" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="8" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="10" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="11" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="12" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>60</v>
       </c>
     </row>
@@ -897,134 +897,134 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="5" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1064,89 +1064,89 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="3" t="s">
         <v>25</v>
       </c>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D8" s="6">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="6" t="s">
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>28</v>
       </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D10" s="6">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6" t="s">
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>29</v>
       </c>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>30</v>
       </c>
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <v>10</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="4" t="s">
         <v>31</v>
       </c>
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="6" t="s">
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>32</v>
       </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D14" s="6">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6" t="s">
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="6" t="s">
+      <c r="D15" s="4">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="D16" s="6">
-        <v>1</v>
-      </c>
-      <c r="E16" s="6" t="s">
+      <c r="D16" s="4">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1167,24 +1167,24 @@
   </cols>
   <sheetData>
     <row r="4" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="8">
         <v>1</v>
       </c>
       <c r="F5" s="9">
@@ -1195,10 +1195,10 @@
       </c>
     </row>
     <row r="6" spans="4:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="8">
         <v>1</v>
       </c>
       <c r="F6" s="9">
@@ -1209,10 +1209,10 @@
       </c>
     </row>
     <row r="7" spans="4:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="8">
         <v>1</v>
       </c>
       <c r="F7" s="9">
@@ -1223,10 +1223,10 @@
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="8">
         <v>1</v>
       </c>
       <c r="F8" s="9">
@@ -1237,10 +1237,10 @@
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="8">
         <v>10</v>
       </c>
       <c r="F9" s="9">
@@ -1251,10 +1251,10 @@
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="8">
         <v>1</v>
       </c>
       <c r="F10" s="9">
@@ -1265,10 +1265,10 @@
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="8">
         <v>1</v>
       </c>
       <c r="F11" s="9">
@@ -1279,10 +1279,10 @@
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="8">
         <v>1</v>
       </c>
       <c r="F12" s="9">
@@ -1296,7 +1296,7 @@
       <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="6">
         <f>SUM(G5:G12)</f>
         <v>430</v>
       </c>

</xml_diff>